<commit_message>
Auto: talaba ma'lumotlari yangilandi (2026-10-20 09:32:19)
</commit_message>
<xml_diff>
--- a/data/Talabalar_Yangilangan_Royxat.xlsx
+++ b/data/Talabalar_Yangilangan_Royxat.xlsx
@@ -41608,9 +41608,9 @@
       </c>
       <c r="V442" s="4" t="inlineStr"/>
       <c r="W442" s="6" t="inlineStr"/>
-      <c r="X442" s="15" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X442" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>
@@ -61480,9 +61480,9 @@
       </c>
       <c r="V26" s="4" t="inlineStr"/>
       <c r="W26" s="6" t="inlineStr"/>
-      <c r="X26" s="15" t="inlineStr">
-        <is>
-          <t>KUTILMOQDA</t>
+      <c r="X26" s="7" t="inlineStr">
+        <is>
+          <t>TASDIQLANDI</t>
         </is>
       </c>
     </row>

</xml_diff>